<commit_message>
v26: logo nuevo, enemigos que huyen, vuelo recto, cámara al objetivo y entrada de cine
- Logo recortado de Jorge con transparencia (imagenes/logo_v3.webp), pasado a PNG con
  Blender (imagen_a_png.py) y separado en SKY y APEX (separar_logo_alfa.mjs).
- Dragones enemigos: radio de giro de 130 m en el Excel (tope del giro total; antes,
  sumando ejes, giraban más que el jugador) y huida hacia delante con maniobras amplias
  cuando los persigues (eses, curvas abiertas, tirabuzón, subidas y picados).
- Controles: Espacio mantenido = vuelo recto con la mira libre, Ctrl izq. = hover,
  F mantenida = cámara al blanco fijado, R = escudo, X = nivelar. En partida, aviso
  antes de cerrar la pestaña (Ctrl+W).
- Entrada de cine al empezar cada misión: vuelo automático con bandas negras, nombre
  de la misión y primeros mensajes de radio; luego se toma el control.
- Textos de Controles, tutorial y Excel actualizados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/sky_apex_stats.xlsx
+++ b/datos/sky_apex_stats.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1088" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1105" uniqueCount="279">
   <si>
     <t>Sky Apex · Stats de las unidades</t>
   </si>
@@ -296,7 +296,7 @@
     <t>armadura_regen</t>
   </si>
   <si>
-    <t>Cargas del escudo (F) al empezar; también es el máximo.</t>
+    <t>Cargas del escudo (R) al empezar; también es el máximo.</t>
   </si>
   <si>
     <t>escudos</t>
@@ -491,6 +491,9 @@
     <t>velocidad</t>
   </si>
   <si>
+    <t>El del giro más cerrado a su velocidad máxima: cuanto más grande, más abiertos sus giros. Si es mayor que el tuyo (Base: 110 m), al perseguirlo puedes cerrar el giro y apuntarle (v26: 130; antes, unos 104 m).</t>
+  </si>
+  <si>
     <t>Distancia de detección</t>
   </si>
   <si>
@@ -507,6 +510,33 @@
   </si>
   <si>
     <t>Puntos al derribarlo</t>
+  </si>
+  <si>
+    <t>Huida (cuando le persigues)</t>
+  </si>
+  <si>
+    <t>Distancia a la que se siente perseguido</t>
+  </si>
+  <si>
+    <t>Con el jugador detrás, apuntándole y más cerca que esto, huye hacia delante con maniobras amplias (eses, curvas abiertas, tirabuzón, subidas y picados).</t>
+  </si>
+  <si>
+    <t>huida_distancia</t>
+  </si>
+  <si>
+    <t>Tiempo de huida (mínimo)</t>
+  </si>
+  <si>
+    <t>Pasado este tiempo (entre el mínimo y el máximo) da la vuelta con una curva abierta y vuelve a atacar.</t>
+  </si>
+  <si>
+    <t>huida_min</t>
+  </si>
+  <si>
+    <t>Tiempo de huida (máximo)</t>
+  </si>
+  <si>
+    <t>huida_max</t>
   </si>
   <si>
     <t>Bola de fuego</t>
@@ -1515,7 +1545,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>224</v>
+        <v>234</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
@@ -1550,7 +1580,7 @@
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -1576,7 +1606,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>225</v>
+        <v>235</v>
       </c>
       <c r="B7" s="16">
         <v>200</v>
@@ -1593,7 +1623,7 @@
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>226</v>
+        <v>236</v>
       </c>
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
@@ -1602,7 +1632,7 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>207</v>
+        <v>217</v>
       </c>
       <c r="B9" s="16">
         <v>1</v>
@@ -1614,12 +1644,12 @@
         <v>154</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>227</v>
+        <v>237</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>165</v>
+        <v>175</v>
       </c>
       <c r="B10" s="16">
         <v>2000</v>
@@ -1631,12 +1661,12 @@
         <v>154</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>228</v>
+        <v>238</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>229</v>
+        <v>239</v>
       </c>
       <c r="B11" s="16">
         <v>0.3</v>
@@ -1645,78 +1675,78 @@
         <v>34</v>
       </c>
       <c r="D11" s="17" t="s">
-        <v>230</v>
+        <v>240</v>
       </c>
       <c r="E11" s="18" t="s">
-        <v>231</v>
+        <v>241</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
-        <v>218</v>
+        <v>228</v>
       </c>
       <c r="B12" s="16">
         <v>800</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>219</v>
+        <v>229</v>
       </c>
       <c r="D12" s="17" t="s">
         <v>154</v>
       </c>
       <c r="E12" s="18" t="s">
-        <v>232</v>
+        <v>242</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
-        <v>221</v>
+        <v>231</v>
       </c>
       <c r="B13" s="16">
         <v>1.72</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>222</v>
+        <v>232</v>
       </c>
       <c r="D13" s="17" t="s">
         <v>154</v>
       </c>
       <c r="E13" s="18" t="s">
-        <v>233</v>
+        <v>243</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
-        <v>234</v>
+        <v>244</v>
       </c>
       <c r="B14" s="16">
         <v>35</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>222</v>
+        <v>232</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>235</v>
+        <v>245</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>236</v>
+        <v>246</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>237</v>
+        <v>247</v>
       </c>
       <c r="B15" s="16">
         <v>50</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>222</v>
+        <v>232</v>
       </c>
       <c r="D15" s="17" t="s">
-        <v>238</v>
+        <v>248</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>239</v>
+        <v>249</v>
       </c>
     </row>
   </sheetData>
@@ -1748,7 +1778,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>240</v>
+        <v>250</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
@@ -1757,7 +1787,7 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>241</v>
+        <v>251</v>
       </c>
       <c r="B2" s="5"/>
       <c r="C2" s="5"/>
@@ -1783,7 +1813,7 @@
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>242</v>
+        <v>252</v>
       </c>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -1809,7 +1839,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>243</v>
+        <v>253</v>
       </c>
       <c r="B7" s="16">
         <v>0.14</v>
@@ -1821,12 +1851,12 @@
         <v>154</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>244</v>
+        <v>254</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>245</v>
+        <v>255</v>
       </c>
       <c r="B8" s="16">
         <v>0.26</v>
@@ -1838,12 +1868,12 @@
         <v>154</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>246</v>
+        <v>256</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>247</v>
+        <v>257</v>
       </c>
       <c r="B9" s="16">
         <v>1000</v>
@@ -1855,24 +1885,24 @@
         <v>154</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>248</v>
+        <v>258</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>171</v>
+        <v>181</v>
       </c>
       <c r="B10" s="16">
         <v>1</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>172</v>
+        <v>182</v>
       </c>
       <c r="D10" s="17" t="s">
         <v>154</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>249</v>
+        <v>259</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -1886,7 +1916,7 @@
         <v>36</v>
       </c>
       <c r="D11" s="17" t="s">
-        <v>250</v>
+        <v>260</v>
       </c>
       <c r="E11" s="18" t="s">
         <v>116</v>
@@ -1911,7 +1941,7 @@
     </row>
     <row r="13" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>251</v>
+        <v>261</v>
       </c>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -1929,7 +1959,7 @@
         <v>72</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>252</v>
+        <v>262</v>
       </c>
       <c r="E14" s="18" t="s">
         <v>136</v>
@@ -1937,7 +1967,7 @@
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>253</v>
+        <v>263</v>
       </c>
       <c r="B15" s="16">
         <v>2000</v>
@@ -1946,15 +1976,15 @@
         <v>53</v>
       </c>
       <c r="D15" s="17" t="s">
-        <v>254</v>
+        <v>264</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>255</v>
+        <v>265</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
-        <v>256</v>
+        <v>266</v>
       </c>
       <c r="B16" s="16">
         <v>1000</v>
@@ -1963,15 +1993,15 @@
         <v>53</v>
       </c>
       <c r="D16" s="17" t="s">
-        <v>257</v>
+        <v>267</v>
       </c>
       <c r="E16" s="18" t="s">
-        <v>258</v>
+        <v>268</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
-        <v>259</v>
+        <v>269</v>
       </c>
       <c r="B17" s="16">
         <v>60</v>
@@ -1980,15 +2010,15 @@
         <v>69</v>
       </c>
       <c r="D17" s="17" t="s">
-        <v>260</v>
+        <v>270</v>
       </c>
       <c r="E17" s="18" t="s">
-        <v>261</v>
+        <v>271</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
-        <v>262</v>
+        <v>272</v>
       </c>
       <c r="B18" s="16">
         <v>600</v>
@@ -1997,15 +2027,15 @@
         <v>53</v>
       </c>
       <c r="D18" s="17" t="s">
-        <v>263</v>
+        <v>273</v>
       </c>
       <c r="E18" s="18" t="s">
-        <v>264</v>
+        <v>274</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
-        <v>265</v>
+        <v>275</v>
       </c>
       <c r="B19" s="16">
         <v>5</v>
@@ -2017,12 +2047,12 @@
         <v>154</v>
       </c>
       <c r="E19" s="18" t="s">
-        <v>266</v>
+        <v>276</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
-        <v>267</v>
+        <v>277</v>
       </c>
       <c r="B20" s="16">
         <v>10</v>
@@ -2034,7 +2064,7 @@
         <v>154</v>
       </c>
       <c r="E20" s="18" t="s">
-        <v>268</v>
+        <v>278</v>
       </c>
     </row>
   </sheetData>
@@ -7832,7 +7862,7 @@
   <sheetPr>
     <tabColor rgb="FF5A6E8A"/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
@@ -7922,121 +7952,121 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>156</v>
+        <v>78</v>
       </c>
       <c r="B8" s="16">
-        <v>2000</v>
+        <v>130</v>
       </c>
       <c r="C8" s="10" t="s">
         <v>53</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="9" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B9" s="16">
-        <v>3500</v>
+        <v>2000</v>
       </c>
       <c r="C9" s="10" t="s">
         <v>53</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B10" s="16">
-        <v>300</v>
+        <v>3500</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>31</v>
+        <v>53</v>
       </c>
       <c r="D10" s="17" t="s">
         <v>154</v>
       </c>
       <c r="E10" s="18" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="B11" s="16">
+        <v>300</v>
+      </c>
+      <c r="C11" s="10" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="11" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="8" t="s">
-        <v>162</v>
-      </c>
-      <c r="B11" s="8"/>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="9" t="s">
+      <c r="D11" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="E11" s="18" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="8" t="s">
         <v>163</v>
       </c>
-      <c r="B12" s="16">
-        <v>10</v>
-      </c>
-      <c r="C12" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="D12" s="17" t="s">
-        <v>154</v>
-      </c>
-      <c r="E12" s="18" t="s">
+      <c r="B12" s="8"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A13" s="13" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="9" t="s">
-        <v>165</v>
-      </c>
       <c r="B13" s="16">
-        <v>1000</v>
+        <v>1800</v>
       </c>
       <c r="C13" s="10" t="s">
         <v>53</v>
       </c>
       <c r="D13" s="17" t="s">
-        <v>154</v>
+        <v>165</v>
       </c>
       <c r="E13" s="18" t="s">
         <v>166</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="9" t="s">
+      <c r="A14" s="13" t="s">
         <v>167</v>
       </c>
       <c r="B14" s="16">
-        <v>1.7</v>
+        <v>10</v>
       </c>
       <c r="C14" s="10" t="s">
         <v>34</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>154</v>
+        <v>168</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="9" t="s">
-        <v>169</v>
+      <c r="A15" s="13" t="s">
+        <v>170</v>
       </c>
       <c r="B15" s="16">
-        <v>2.9</v>
+        <v>18</v>
       </c>
       <c r="C15" s="10" t="s">
         <v>34</v>
@@ -8045,44 +8075,44 @@
         <v>154</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="9" t="s">
         <v>171</v>
       </c>
-      <c r="B16" s="16">
-        <v>2.2</v>
-      </c>
-      <c r="C16" s="10" t="s">
+    </row>
+    <row r="16" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="8" t="s">
         <v>172</v>
       </c>
-      <c r="D16" s="17" t="s">
+      <c r="B16" s="8"/>
+      <c r="C16" s="8"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A17" s="9" t="s">
+        <v>173</v>
+      </c>
+      <c r="B17" s="16">
+        <v>10</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="D17" s="17" t="s">
         <v>154</v>
       </c>
-      <c r="E16" s="18" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="17" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="8" t="s">
+      <c r="E17" s="18" t="s">
         <v>174</v>
       </c>
-      <c r="B17" s="8"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="8"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
         <v>175</v>
       </c>
       <c r="B18" s="16">
-        <v>30</v>
+        <v>1000</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>31</v>
+        <v>53</v>
       </c>
       <c r="D18" s="17" t="s">
         <v>154</v>
@@ -8093,16 +8123,16 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
-        <v>54</v>
+        <v>177</v>
       </c>
       <c r="B19" s="16">
-        <v>4</v>
+        <v>1.7</v>
       </c>
       <c r="C19" s="10" t="s">
         <v>34</v>
       </c>
       <c r="D19" s="17" t="s">
-        <v>177</v>
+        <v>154</v>
       </c>
       <c r="E19" s="18" t="s">
         <v>178</v>
@@ -8113,10 +8143,10 @@
         <v>179</v>
       </c>
       <c r="B20" s="16">
-        <v>500</v>
+        <v>2.9</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>53</v>
+        <v>34</v>
       </c>
       <c r="D20" s="17" t="s">
         <v>154</v>
@@ -8130,137 +8160,215 @@
         <v>181</v>
       </c>
       <c r="B21" s="16">
-        <v>2000</v>
+        <v>2.2</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>53</v>
+        <v>182</v>
       </c>
       <c r="D21" s="17" t="s">
         <v>154</v>
       </c>
       <c r="E21" s="18" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="9" t="s">
         <v>183</v>
       </c>
-      <c r="B22" s="16">
-        <v>60</v>
-      </c>
-      <c r="C22" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="D22" s="17" t="s">
-        <v>154</v>
-      </c>
-      <c r="E22" s="18" t="s">
+    </row>
+    <row r="22" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A22" s="8" t="s">
         <v>184</v>
       </c>
+      <c r="B22" s="8"/>
+      <c r="C22" s="8"/>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
         <v>185</v>
       </c>
       <c r="B23" s="16">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D23" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="E23" s="18" t="s">
         <v>186</v>
-      </c>
-      <c r="E23" s="18" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B24" s="16">
+        <v>4</v>
+      </c>
+      <c r="C24" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="D24" s="17" t="s">
+        <v>187</v>
+      </c>
+      <c r="E24" s="18" t="s">
         <v>188</v>
-      </c>
-      <c r="B24" s="16">
-        <v>1152</v>
-      </c>
-      <c r="C24" s="10" t="s">
-        <v>72</v>
-      </c>
-      <c r="D24" s="17" t="s">
-        <v>154</v>
-      </c>
-      <c r="E24" s="18" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="B25" s="16">
+        <v>500</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="D25" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="E25" s="18" t="s">
         <v>190</v>
       </c>
-      <c r="B25" s="16">
-        <v>30</v>
-      </c>
-      <c r="C25" s="10" t="s">
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" s="9" t="s">
         <v>191</v>
       </c>
-      <c r="D25" s="17" t="s">
+      <c r="B26" s="16">
+        <v>2000</v>
+      </c>
+      <c r="C26" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="D26" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="E26" s="18" t="s">
         <v>192</v>
       </c>
-      <c r="E25" s="18" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="26" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="8" t="s">
-        <v>194</v>
-      </c>
-      <c r="B26" s="8"/>
-      <c r="C26" s="8"/>
-      <c r="D26" s="8"/>
-      <c r="E26" s="8"/>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="9" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B27" s="16">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D27" s="17" t="s">
         <v>154</v>
       </c>
       <c r="E27" s="18" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="9" t="s">
+        <v>195</v>
+      </c>
+      <c r="B28" s="16">
+        <v>20</v>
+      </c>
+      <c r="C28" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="D28" s="17" t="s">
+        <v>196</v>
+      </c>
+      <c r="E28" s="18" t="s">
         <v>197</v>
       </c>
-      <c r="B28" s="16">
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" s="9" t="s">
+        <v>198</v>
+      </c>
+      <c r="B29" s="16">
+        <v>1152</v>
+      </c>
+      <c r="C29" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="D29" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="E29" s="18" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" s="9" t="s">
+        <v>200</v>
+      </c>
+      <c r="B30" s="16">
+        <v>30</v>
+      </c>
+      <c r="C30" s="10" t="s">
+        <v>201</v>
+      </c>
+      <c r="D30" s="17" t="s">
+        <v>202</v>
+      </c>
+      <c r="E30" s="18" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="31" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="B31" s="8"/>
+      <c r="C31" s="8"/>
+      <c r="D31" s="8"/>
+      <c r="E31" s="8"/>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" s="9" t="s">
+        <v>205</v>
+      </c>
+      <c r="B32" s="16">
+        <v>25</v>
+      </c>
+      <c r="C32" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="D32" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="E32" s="18" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="B33" s="16">
         <v>50</v>
       </c>
-      <c r="C28" s="10" t="s">
+      <c r="C33" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="D28" s="17" t="s">
+      <c r="D33" s="17" t="s">
         <v>154</v>
       </c>
-      <c r="E28" s="18" t="s">
-        <v>198</v>
+      <c r="E33" s="18" t="s">
+        <v>208</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A11:E11"/>
-    <mergeCell ref="A17:E17"/>
-    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="A12:E12"/>
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="A22:E22"/>
+    <mergeCell ref="A31:E31"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -8284,7 +8392,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>199</v>
+        <v>209</v>
       </c>
       <c r="B1" s="4"/>
       <c r="C1" s="4"/>
@@ -8319,7 +8427,7 @@
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -8345,7 +8453,7 @@
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
-        <v>201</v>
+        <v>211</v>
       </c>
       <c r="B7" s="16">
         <v>100</v>
@@ -8362,24 +8470,24 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>202</v>
+        <v>212</v>
       </c>
       <c r="B8" s="16">
         <v>1</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>203</v>
+        <v>213</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>204</v>
+        <v>214</v>
       </c>
       <c r="E8" s="18" t="s">
-        <v>205</v>
+        <v>215</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>206</v>
+        <v>216</v>
       </c>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
@@ -8388,7 +8496,7 @@
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
-        <v>207</v>
+        <v>217</v>
       </c>
       <c r="B10" s="16">
         <v>3</v>
@@ -8400,12 +8508,12 @@
         <v>154</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>208</v>
+        <v>218</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="9" t="s">
-        <v>165</v>
+        <v>175</v>
       </c>
       <c r="B11" s="16">
         <v>1500</v>
@@ -8417,12 +8525,12 @@
         <v>154</v>
       </c>
       <c r="E11" s="18" t="s">
-        <v>209</v>
+        <v>219</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
-        <v>210</v>
+        <v>220</v>
       </c>
       <c r="B12" s="16">
         <v>5</v>
@@ -8434,12 +8542,12 @@
         <v>154</v>
       </c>
       <c r="E12" s="18" t="s">
-        <v>211</v>
+        <v>221</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="9" t="s">
-        <v>212</v>
+        <v>222</v>
       </c>
       <c r="B13" s="16">
         <v>0.12</v>
@@ -8451,12 +8559,12 @@
         <v>154</v>
       </c>
       <c r="E13" s="18" t="s">
-        <v>213</v>
+        <v>223</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
-        <v>214</v>
+        <v>224</v>
       </c>
       <c r="B14" s="16">
         <v>2.2</v>
@@ -8468,12 +8576,12 @@
         <v>154</v>
       </c>
       <c r="E14" s="18" t="s">
-        <v>215</v>
+        <v>225</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="9" t="s">
-        <v>216</v>
+        <v>226</v>
       </c>
       <c r="B15" s="16">
         <v>3.6</v>
@@ -8485,41 +8593,41 @@
         <v>154</v>
       </c>
       <c r="E15" s="18" t="s">
-        <v>217</v>
+        <v>227</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
-        <v>218</v>
+        <v>228</v>
       </c>
       <c r="B16" s="16">
         <v>1100</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>219</v>
+        <v>229</v>
       </c>
       <c r="D16" s="17" t="s">
         <v>154</v>
       </c>
       <c r="E16" s="18" t="s">
-        <v>220</v>
+        <v>230</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
-        <v>221</v>
+        <v>231</v>
       </c>
       <c r="B17" s="16">
         <v>2</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>222</v>
+        <v>232</v>
       </c>
       <c r="D17" s="17" t="s">
         <v>154</v>
       </c>
       <c r="E17" s="18" t="s">
-        <v>223</v>
+        <v>233</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
v30: arreglos de la galería de enemigos
- Apuntado: la mira saltaba al punto de interceptación viejo de un dragón al
  apuntar a cualquier unidad nueva (cabeza girada, cámara rara, llamarada a
  otro lado). Impactos en la superficie de las cápsulas y todo apunta al
  centro de las unidades (targetCenter).
- Sierpe rehecha desde el FBX original: patas bien, aletas dorsales, patas
  rígidas con su hombro (pesos de los huesos) y patrulla circular amplia.
- Superdirigible de 1000 m con dos chorros de motor arcano.
- Bola guiada con parábola contra tierra y mar; cuenta si cae junto al blanco.
- stats_excel.mjs --poner unidad.clave=valor.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/sky_apex_stats.xlsx
+++ b/datos/sky_apex_stats.xlsx
@@ -1003,7 +1003,7 @@
     <t>Se puede dañar aunque queden torretas; al caer, caen todas.</t>
   </si>
   <si>
-    <t>Jorge: 500 m como mínimo.</t>
+    <t>Jorge: 500 m como mínimo (v29) y luego el doble (v30). Las torretas no cambian de tamaño: quedan más separadas.</t>
   </si>
   <si>
     <t>Altura mínima de vuelo</t>
@@ -1093,7 +1093,7 @@
     <t>Radio del círculo</t>
   </si>
   <si>
-    <t>En vuelo circular (en la galería, con el panel de pruebas).</t>
+    <t>En vuelo circular: su patrulla (en la galería, sobre todo el campo).</t>
   </si>
   <si>
     <t>radio_circulo</t>
@@ -3157,7 +3157,7 @@
         <v>318</v>
       </c>
       <c r="B8" s="16">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="C8" s="10" t="s">
         <v>54</v>
@@ -3552,7 +3552,7 @@
         <v>354</v>
       </c>
       <c r="B11" s="16">
-        <v>2500</v>
+        <v>3500</v>
       </c>
       <c r="C11" s="10" t="s">
         <v>54</v>

</xml_diff>

<commit_message>
v31: fijar y apuntar más cómodo; el superdirigible cae en llamas
- Círculo de adelanto solo con blancos a más de 150 km/h.
- Fijar: primero lo más cercano a la mira; apuntando al mismo sitio, cada
  clic pasa al siguiente más cercano.
- Bola guiada: fijado en 2 s (Excel y código).
- Superdirigible: barra de vida grande bajo el casco con las torretas que
  quedan; al destruirlo cae ennegrecido y en llamas con estela de humo y se
  estrella contra el suelo.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/sky_apex_stats.xlsx
+++ b/datos/sky_apex_stats.xlsx
@@ -370,7 +370,7 @@
     <t>guiado_alcance</t>
   </si>
   <si>
-    <t>Segundos con la mira en el círculo rojo hasta que sale.</t>
+    <t>Segundos con la mira en el círculo rojo hasta que sale (v31: 2, antes 3).</t>
   </si>
   <si>
     <t>guiado_fijado</t>
@@ -4665,23 +4665,23 @@
       </c>
       <c r="C23" s="11">
         <f>Base!B23</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D23" s="12">
         <f>'Alientormenta'!B23</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E23" s="12">
         <f>'Abrasanubes'!B23</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F23" s="12">
         <f>'Ventoscuro'!B23</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G23" s="12">
         <f>'Fulgor'!B23</f>
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="24" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -5551,7 +5551,7 @@
         <v>55</v>
       </c>
       <c r="B23" s="16">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C23" s="10" t="s">
         <v>35</v>
@@ -6386,14 +6386,14 @@
       </c>
       <c r="B23" s="16">
         <f>Base!B23</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C23" s="10" t="s">
         <v>35</v>
       </c>
       <c r="D23" s="10">
         <f>Base!B23</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E23" s="19">
         <f>IF(D23=0,"",B23/D23-1)</f>
@@ -7393,14 +7393,14 @@
       </c>
       <c r="B23" s="16">
         <f>Base!B23</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C23" s="10" t="s">
         <v>35</v>
       </c>
       <c r="D23" s="10">
         <f>Base!B23</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E23" s="19">
         <f>IF(D23=0,"",B23/D23-1)</f>
@@ -8400,14 +8400,14 @@
       </c>
       <c r="B23" s="16">
         <f>Base!B23</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C23" s="10" t="s">
         <v>35</v>
       </c>
       <c r="D23" s="10">
         <f>Base!B23</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E23" s="19">
         <f>IF(D23=0,"",B23/D23-1)</f>
@@ -9407,14 +9407,14 @@
       </c>
       <c r="B23" s="16">
         <f>Base!B23</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C23" s="10" t="s">
         <v>35</v>
       </c>
       <c r="D23" s="10">
         <f>Base!B23</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E23" s="19">
         <f>IF(D23=0,"",B23/D23-1)</f>

</xml_diff>

<commit_message>
v33: esquiva de 30 m en 1,5 s y alas en picado sin cruzarse
- Esquiva por defecto: 30 m en 1,5 s (Excel y código).
- Picado: el brazo va menos atrás y los dedos cierran el abanico hacia la cola;
  las alas ya no se cruzan por detrás. Ventoscuro, con su propio pliegue.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datos/sky_apex_stats.xlsx
+++ b/datos/sky_apex_stats.xlsx
@@ -5252,23 +5252,23 @@
       </c>
       <c r="C45" s="11">
         <f>Base!B45</f>
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="D45" s="12">
         <f>'Alientormenta'!B45</f>
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="E45" s="12">
         <f>'Abrasanubes'!B45</f>
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F45" s="12">
         <f>'Ventoscuro'!B45</f>
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="G45" s="12">
         <f>'Fulgor'!B45</f>
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
@@ -5280,23 +5280,23 @@
       </c>
       <c r="C46" s="11">
         <f>Base!B46</f>
-        <v>0.6</v>
+        <v>1.5</v>
       </c>
       <c r="D46" s="12">
         <f>'Alientormenta'!B46</f>
-        <v>0.6</v>
+        <v>1.5</v>
       </c>
       <c r="E46" s="12">
         <f>'Abrasanubes'!B46</f>
-        <v>0.6</v>
+        <v>1.5</v>
       </c>
       <c r="F46" s="12">
         <f>'Ventoscuro'!B46</f>
-        <v>0.6</v>
+        <v>1.5</v>
       </c>
       <c r="G46" s="12">
         <f>'Fulgor'!B46</f>
-        <v>0.6</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
@@ -6056,7 +6056,7 @@
         <v>81</v>
       </c>
       <c r="B45" s="16">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="C45" s="10" t="s">
         <v>54</v>
@@ -6073,7 +6073,7 @@
         <v>82</v>
       </c>
       <c r="B46" s="16">
-        <v>0.6</v>
+        <v>1.5</v>
       </c>
       <c r="C46" s="10" t="s">
         <v>35</v>
@@ -7139,14 +7139,14 @@
       </c>
       <c r="B45" s="16">
         <f>Base!B45</f>
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="C45" s="10" t="s">
         <v>54</v>
       </c>
       <c r="D45" s="10">
         <f>Base!B45</f>
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="E45" s="19">
         <f>IF(D45=0,"",B45/D45-1)</f>
@@ -7165,14 +7165,14 @@
       </c>
       <c r="B46" s="16">
         <f>Base!B46</f>
-        <v>0.6</v>
+        <v>1.5</v>
       </c>
       <c r="C46" s="10" t="s">
         <v>35</v>
       </c>
       <c r="D46" s="10">
         <f>Base!B46</f>
-        <v>0.6</v>
+        <v>1.5</v>
       </c>
       <c r="E46" s="19">
         <f>IF(D46=0,"",B46/D46-1)</f>
@@ -8262,14 +8262,14 @@
       </c>
       <c r="B45" s="16">
         <f>Base!B45</f>
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="C45" s="10" t="s">
         <v>54</v>
       </c>
       <c r="D45" s="10">
         <f>Base!B45</f>
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="E45" s="19">
         <f>IF(D45=0,"",B45/D45-1)</f>
@@ -8288,14 +8288,14 @@
       </c>
       <c r="B46" s="16">
         <f>Base!B46</f>
-        <v>0.6</v>
+        <v>1.5</v>
       </c>
       <c r="C46" s="10" t="s">
         <v>35</v>
       </c>
       <c r="D46" s="10">
         <f>Base!B46</f>
-        <v>0.6</v>
+        <v>1.5</v>
       </c>
       <c r="E46" s="19">
         <f>IF(D46=0,"",B46/D46-1)</f>
@@ -9385,14 +9385,14 @@
       </c>
       <c r="B45" s="16">
         <f>Base!B45</f>
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="C45" s="10" t="s">
         <v>54</v>
       </c>
       <c r="D45" s="10">
         <f>Base!B45</f>
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="E45" s="19">
         <f>IF(D45=0,"",B45/D45-1)</f>
@@ -9411,14 +9411,14 @@
       </c>
       <c r="B46" s="16">
         <f>Base!B46</f>
-        <v>0.6</v>
+        <v>1.5</v>
       </c>
       <c r="C46" s="10" t="s">
         <v>35</v>
       </c>
       <c r="D46" s="10">
         <f>Base!B46</f>
-        <v>0.6</v>
+        <v>1.5</v>
       </c>
       <c r="E46" s="19">
         <f>IF(D46=0,"",B46/D46-1)</f>
@@ -10508,14 +10508,14 @@
       </c>
       <c r="B45" s="16">
         <f>Base!B45</f>
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="C45" s="10" t="s">
         <v>54</v>
       </c>
       <c r="D45" s="10">
         <f>Base!B45</f>
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="E45" s="19">
         <f>IF(D45=0,"",B45/D45-1)</f>
@@ -10534,14 +10534,14 @@
       </c>
       <c r="B46" s="16">
         <f>Base!B46</f>
-        <v>0.6</v>
+        <v>1.5</v>
       </c>
       <c r="C46" s="10" t="s">
         <v>35</v>
       </c>
       <c r="D46" s="10">
         <f>Base!B46</f>
-        <v>0.6</v>
+        <v>1.5</v>
       </c>
       <c r="E46" s="19">
         <f>IF(D46=0,"",B46/D46-1)</f>

</xml_diff>